<commit_message>
Drop the YouTube hours-watched rate to $0.50 per hour
Was $1.00. Changed in the store's defaults, the spreadsheet generator,
the docs, and the test expectations, and the .xlsx is rebuilt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxionAVqcMNjbxNZALQNHW
</commit_message>
<xml_diff>
--- a/social-media-bonus-tracker.xlsx
+++ b/social-media-bonus-tracker.xlsx
@@ -720,7 +720,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Google positive reviews $1.50 · YouTube hours watched $1.00 per hour.</t>
+          <t>Google positive reviews $1.50 · YouTube hours watched $0.50 per hour.</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
         <v/>
       </c>
       <c r="C9" s="17" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Google positive reviews $1.50, YouTube hours watched $1.00 per hour.</t>
+          <t xml:space="preserve">  Google positive reviews $1.50, YouTube hours watched $0.50 per hour.</t>
         </is>
       </c>
     </row>

</xml_diff>